<commit_message>
chore(balance): finalize economy-contract README, pin docs to LF, stop shadow-overlay churn
</commit_message>
<xml_diff>
--- a/docs/archive/balance-v1.xlsx
+++ b/docs/archive/balance-v1.xlsx
@@ -1,26 +1,3 @@
-
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
-  </bookViews>
-  <sheets>
-    <sheet name="Read Me" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Crops" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Levels" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Orders &amp; Sanity" sheetId="4" state="visible" r:id="rId6"/>
-  </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
-</workbook>
-</file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="72">
@@ -241,532 +218,6 @@
     <t xml:space="preserve">Green = pulls live from the Crops sheet. Change a blue crop number and everything here follows.</t>
   </si>
 </sst>
-</file>
-
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="0.00"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-  </numFmts>
-  <fonts count="9">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <i val="true"/>
-      <sz val="10"/>
-      <color rgb="FF555555"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF008000"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-  </fonts>
-  <fills count="4">
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFDDE8D9"/>
-        <bgColor rgb="FFCCFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-  </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-  </cellXfs>
-  <cellStyles count="6">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
-  </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFDDE8D9"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF555555"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
-  <dimension ref="A1:A20"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>